<commit_message>
Complete task13 listing lifecycle handoff
</commit_message>
<xml_diff>
--- a/data/samples/listing_rules.xlsx
+++ b/data/samples/listing_rules.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -508,7 +508,6 @@
       <c r="I2" t="n">
         <v>1</v>
       </c>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -550,7 +549,383 @@
       <c r="I3" t="n">
         <v>5</v>
       </c>
-      <c r="J3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>LIST-全平台艾莎A上架</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>全平台艾莎A上架</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>艾莎</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>allow_online</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LIST-蚂蚁艾莎A</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>蚂蚁艾莎A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>艾莎</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>蚂蚁</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>allow_online</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LIST-蚂蚁艾莎A下架</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>蚂蚁艾莎A下架</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>艾莎</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>蚂蚁</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>set_offline</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LIST-蚂蚁E级上架</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>蚂蚁E级上架</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>蚂蚁</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>allow_online</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LIST-E级蚂蚁下架</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>E级蚂蚁下架</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>蚂蚁</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>set_offline</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LIST-蚂蚁艾莎下架</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>蚂蚁艾莎下架</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>艾莎</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>蚂蚁</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>set_offline</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LIST-艾莎B级上架</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>艾莎B级上架</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>艾莎</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>蚂蚁</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>allow_online</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LIST-蚂蚁B级下架</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>蚂蚁B级下架</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>蚂蚁</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>set_offline</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>